<commit_message>
Reprocess data from 20241204
</commit_message>
<xml_diff>
--- a/data/VMP/20241204/Level0/Logbook_Zug_20241204.xlsx
+++ b/data/VMP/20241204/Level0/Logbook_Zug_20241204.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unils-my.sharepoint.com/personal/tomy_doda_unil_ch/Documents/Fieldwork/Lake_Zug/20241204_Campaign/Data/VMP/Profiles_20241204/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tdoda\OneDrive - Université de Lausanne\Projects\3-Zug\turbulence-lakezug\data\VMP\20241204\Level0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{46C9F045-E8EE-4D12-BB21-4E4335B67692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02BC6873-06E4-49AB-9CD7-9A474F892FB5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F97EAE30-667A-4A71-BFDC-08A402DAEF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1140" yWindow="1140" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Logbook_Zug" sheetId="1" r:id="rId1"/>
@@ -187,7 +187,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -220,6 +220,13 @@
     <font>
       <sz val="11"/>
       <color theme="2" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -334,7 +341,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -444,28 +451,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Excel Built-in Bad" xfId="2" xr:uid="{88070955-E48E-4170-B9FA-1C6ECF97D977}"/>
@@ -756,32 +760,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z22"/>
-  <sheetFormatPr defaultColWidth="17.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Z19"/>
+  <sheetFormatPr defaultColWidth="17.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="10.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="10.1796875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="17.7265625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="13.81640625" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" style="6" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" style="5" customWidth="1"/>
-    <col min="7" max="7" width="14.5703125" style="15" customWidth="1"/>
-    <col min="8" max="8" width="20.5703125" style="5" customWidth="1"/>
-    <col min="9" max="9" width="13.5703125" style="5" customWidth="1"/>
-    <col min="10" max="11" width="14.5703125" style="5" customWidth="1"/>
-    <col min="12" max="12" width="15.42578125" style="5" customWidth="1"/>
-    <col min="13" max="13" width="10.85546875" style="4" customWidth="1"/>
-    <col min="14" max="14" width="7.7109375" style="4" customWidth="1"/>
-    <col min="15" max="18" width="17.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="19.54296875" style="5" customWidth="1"/>
+    <col min="7" max="7" width="14.54296875" style="15" customWidth="1"/>
+    <col min="8" max="8" width="20.54296875" style="5" customWidth="1"/>
+    <col min="9" max="9" width="13.54296875" style="5" customWidth="1"/>
+    <col min="10" max="11" width="14.54296875" style="5" customWidth="1"/>
+    <col min="12" max="12" width="15.453125" style="5" customWidth="1"/>
+    <col min="13" max="13" width="10.81640625" style="4" customWidth="1"/>
+    <col min="14" max="14" width="7.7265625" style="4" customWidth="1"/>
+    <col min="15" max="18" width="17.7265625" style="2" customWidth="1"/>
     <col min="19" max="19" width="11" style="2" customWidth="1"/>
-    <col min="20" max="20" width="11.85546875" style="2" customWidth="1"/>
-    <col min="21" max="21" width="9.28515625" style="2" customWidth="1"/>
-    <col min="22" max="23" width="9.42578125" style="2" customWidth="1"/>
-    <col min="24" max="24" width="9.28515625" style="2" customWidth="1"/>
+    <col min="20" max="20" width="11.81640625" style="2" customWidth="1"/>
+    <col min="21" max="21" width="9.26953125" style="2" customWidth="1"/>
+    <col min="22" max="23" width="9.453125" style="2" customWidth="1"/>
+    <col min="24" max="24" width="9.26953125" style="2" customWidth="1"/>
     <col min="25" max="25" width="14" style="2" customWidth="1"/>
-    <col min="26" max="26" width="74.42578125" style="5" customWidth="1"/>
+    <col min="26" max="26" width="74.453125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" s="1" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
         <v>2</v>
       </c>
@@ -861,7 +865,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:26" s="40" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" s="40" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="36" t="s">
         <v>25</v>
       </c>
@@ -939,7 +943,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>30</v>
       </c>
@@ -1004,14 +1008,14 @@
       <c r="X3" s="8">
         <v>191</v>
       </c>
-      <c r="Y3" s="46" t="s">
+      <c r="Y3" s="42" t="s">
         <v>46</v>
       </c>
       <c r="Z3" s="8" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:26" s="20" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" s="20" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="17" t="s">
         <v>32</v>
       </c>
@@ -1089,7 +1093,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:26" s="21" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" s="21" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="24" t="s">
         <v>34</v>
       </c>
@@ -1167,7 +1171,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:26" s="22" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="27" t="s">
         <v>35</v>
       </c>
@@ -1245,7 +1249,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:26" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" s="23" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="30" t="s">
         <v>37</v>
       </c>
@@ -1315,75 +1319,75 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:26" s="44" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="41" t="s">
+    <row r="8" spans="1:26" s="47" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="41">
+      <c r="B8" s="44">
         <v>1</v>
       </c>
-      <c r="C8" s="41" t="s">
+      <c r="C8" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="42">
+      <c r="D8" s="45">
         <v>45630</v>
       </c>
-      <c r="E8" s="41">
+      <c r="E8" s="44">
         <v>14</v>
       </c>
-      <c r="F8" s="41">
+      <c r="F8" s="44">
         <v>45</v>
       </c>
-      <c r="G8" s="41">
+      <c r="G8" s="44">
         <v>15</v>
       </c>
-      <c r="H8" s="41">
+      <c r="H8" s="44">
         <v>45</v>
       </c>
-      <c r="I8" s="41"/>
-      <c r="J8" s="41"/>
-      <c r="K8" s="41"/>
-      <c r="L8" s="41"/>
-      <c r="M8" s="43">
+      <c r="I8" s="44"/>
+      <c r="J8" s="44"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="44"/>
+      <c r="M8" s="46">
         <v>680217</v>
       </c>
-      <c r="N8" s="43">
+      <c r="N8" s="46">
         <v>218560</v>
       </c>
-      <c r="O8" s="41" t="s">
+      <c r="O8" s="44" t="s">
         <v>36</v>
       </c>
-      <c r="P8" s="41"/>
-      <c r="Q8" s="41" t="s">
-        <v>28</v>
-      </c>
-      <c r="R8" s="41">
-        <v>28</v>
-      </c>
-      <c r="S8" s="41">
+      <c r="P8" s="44"/>
+      <c r="Q8" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="R8" s="44">
+        <v>28</v>
+      </c>
+      <c r="S8" s="44">
         <v>1699</v>
       </c>
-      <c r="T8" s="41">
+      <c r="T8" s="44">
         <v>1704</v>
       </c>
-      <c r="U8" s="41">
+      <c r="U8" s="44">
         <v>2020</v>
       </c>
-      <c r="V8" s="41">
+      <c r="V8" s="44">
         <v>2080</v>
       </c>
-      <c r="W8" s="41">
+      <c r="W8" s="44">
         <v>190</v>
       </c>
-      <c r="X8" s="41">
+      <c r="X8" s="44">
         <v>191</v>
       </c>
-      <c r="Y8" s="41"/>
-      <c r="Z8" s="41" t="s">
+      <c r="Y8" s="44"/>
+      <c r="Z8" s="44" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:26" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" s="16" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="33" t="s">
         <v>38</v>
       </c>
@@ -1459,48 +1463,22 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="E10" s="15"/>
-      <c r="Y10" s="45"/>
+      <c r="Y10" s="41"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="Y11" s="45"/>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="Y11" s="41"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="Y12" s="45"/>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="Y12" s="41"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="Y13" s="45"/>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="Y13" s="41"/>
     </row>
-    <row r="17" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J17" s="47"/>
-      <c r="K17" s="47"/>
-      <c r="L17" s="47"/>
-    </row>
-    <row r="18" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J18" s="47"/>
-      <c r="K18" s="47"/>
-      <c r="L18" s="47"/>
-    </row>
-    <row r="19" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J19" s="47"/>
-      <c r="K19" s="48"/>
-      <c r="L19" s="48"/>
-    </row>
-    <row r="20" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J20" s="47"/>
-      <c r="K20" s="47"/>
-      <c r="L20" s="47"/>
-    </row>
-    <row r="21" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J21" s="47"/>
-      <c r="K21" s="47"/>
-      <c r="L21" s="47"/>
-    </row>
-    <row r="22" spans="10:12" x14ac:dyDescent="0.25">
-      <c r="J22" s="47"/>
-      <c r="K22" s="47"/>
-      <c r="L22" s="47"/>
+    <row r="19" spans="11:12" x14ac:dyDescent="0.35">
+      <c r="K19" s="43"/>
+      <c r="L19" s="43"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>